<commit_message>
calc metric for gemma4 in one prompt. Conclusion - not great
</commit_message>
<xml_diff>
--- a/src/results/llm/single_prompt_testing_01/responses/results_for_presentation_single_prompt.xlsx
+++ b/src/results/llm/single_prompt_testing_01/responses/results_for_presentation_single_prompt.xlsx
@@ -8,27 +8,35 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\repos\Using-LLM-for-automated-feedback-generation-on-a-bachelor-thesis\src\results\llm\single_prompt_testing_01\responses\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FBF0DF1D-882F-4AD3-978C-2E5835E787BB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8AE37CFA-752D-40AC-A8CF-ADFE1C4F1433}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="15" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
-  <si>
-    <t>gemma4-26b-q4 vs humanx</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="13">
   <si>
     <t>human1</t>
   </si>
@@ -52,14 +60,37 @@
   </si>
   <si>
     <t>CohenKappa</t>
+  </si>
+  <si>
+    <t>gemma4-26b-q4 vs humanx when 'feeback' field absence caused parsing error</t>
+  </si>
+  <si>
+    <t>gemma4-26b-q4 vs humanx when 'feeback' field was optional</t>
+  </si>
+  <si>
+    <t>20 cases which is</t>
+  </si>
+  <si>
+    <t>37 cases which is</t>
+  </si>
+  <si>
+    <t>percentage not parsed</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -87,9 +118,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -372,91 +407,228 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F5"/>
+  <dimension ref="A1:H11"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="20.7109375" customWidth="1"/>
-    <col min="3" max="3" width="16.42578125" customWidth="1"/>
-    <col min="4" max="4" width="14.7109375" customWidth="1"/>
-    <col min="5" max="5" width="11.7109375" customWidth="1"/>
-    <col min="6" max="6" width="13.28515625" customWidth="1"/>
+    <col min="2" max="2" width="20.7109375" style="2" customWidth="1"/>
+    <col min="3" max="3" width="16.42578125" style="2" customWidth="1"/>
+    <col min="4" max="4" width="14.7109375" style="2" customWidth="1"/>
+    <col min="5" max="5" width="11.7109375" style="2" customWidth="1"/>
+    <col min="6" max="6" width="13.28515625" style="2" customWidth="1"/>
+    <col min="8" max="8" width="24.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
       <c r="D1" s="1"/>
       <c r="E1" s="1"/>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="B2" t="s">
+      <c r="F1" s="1"/>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="B2" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="C2" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="C2" t="s">
+      <c r="D2" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="D2" t="s">
+      <c r="E2" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="E2" t="s">
+      <c r="F2" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="F2" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
+        <v>0</v>
+      </c>
+      <c r="B3" s="2">
+        <v>0.86513994910941405</v>
+      </c>
+      <c r="C3" s="2">
+        <v>0.46703296703296698</v>
+      </c>
+      <c r="D3" s="2">
+        <v>0.60660124888492395</v>
+      </c>
+      <c r="E3" s="2">
+        <v>0.63510840476282804</v>
+      </c>
+      <c r="F3" s="2">
+        <v>0.32199138227499802</v>
+      </c>
+      <c r="H3" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
+      <c r="B4" s="2">
+        <v>0.631043256997455</v>
+      </c>
+      <c r="C4" s="2">
+        <v>0.43508771929824502</v>
+      </c>
+      <c r="D4" s="2">
+        <v>0.515057113187954</v>
+      </c>
+      <c r="E4" s="2">
+        <v>0.59857688879275095</v>
+      </c>
+      <c r="F4" s="2">
+        <v>0.214548512561757</v>
+      </c>
+      <c r="H4" s="3">
+        <f>(37/64)*100</f>
+        <v>57.8125</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
         <v>2</v>
       </c>
-      <c r="B4">
-        <v>0.61946902654867197</v>
-      </c>
-      <c r="C4">
-        <v>0.24561403508771901</v>
-      </c>
-      <c r="D4">
-        <v>0.35175879396984899</v>
-      </c>
-      <c r="E4">
-        <v>0.51817768549348198</v>
-      </c>
-      <c r="F4">
-        <v>0.116627434196447</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
+      <c r="B5" s="2">
+        <v>0.87022900763358702</v>
+      </c>
+      <c r="C5" s="2">
+        <v>0.42857142857142799</v>
+      </c>
+      <c r="D5" s="2">
+        <v>0.57430730478589398</v>
+      </c>
+      <c r="E5" s="2">
+        <v>0.58288290299729795</v>
+      </c>
+      <c r="F5" s="2">
+        <v>0.24909747292418699</v>
+      </c>
+      <c r="H5" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A7" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B7" s="1"/>
+      <c r="C7" s="1"/>
+      <c r="D7" s="1"/>
+      <c r="E7" s="1"/>
+      <c r="F7" s="1"/>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="B8" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="B5">
-        <v>0.86725663716814105</v>
-      </c>
-      <c r="C5">
-        <v>0.24561403508771901</v>
-      </c>
-      <c r="D5">
-        <v>0.3828125</v>
-      </c>
-      <c r="E5">
-        <v>0.46697443181818099</v>
-      </c>
-      <c r="F5">
-        <v>0.131122185942601</v>
+      <c r="C8" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="E8" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="F8" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>0</v>
+      </c>
+      <c r="B9" s="2">
+        <v>0.83447098976109202</v>
+      </c>
+      <c r="C9" s="2">
+        <v>0.67170329670329598</v>
+      </c>
+      <c r="D9" s="2">
+        <v>0.74429223744292194</v>
+      </c>
+      <c r="E9" s="2">
+        <v>0.72187778240661304</v>
+      </c>
+      <c r="F9" s="2">
+        <v>0.451287120202845</v>
+      </c>
+      <c r="H9" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>1</v>
+      </c>
+      <c r="B10" s="2">
+        <v>0.639931740614334</v>
+      </c>
+      <c r="C10" s="2">
+        <v>0.65789473684210498</v>
+      </c>
+      <c r="D10" s="2">
+        <v>0.64878892733563998</v>
+      </c>
+      <c r="E10" s="2">
+        <v>0.66530355457691004</v>
+      </c>
+      <c r="F10" s="2">
+        <v>0.330723263960436</v>
+      </c>
+      <c r="H10" s="3">
+        <f>(20/64)*100</f>
+        <v>31.25</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>2</v>
+      </c>
+      <c r="B11" s="2">
+        <v>0.86177474402730303</v>
+      </c>
+      <c r="C11" s="2">
+        <v>0.63283208020050097</v>
+      </c>
+      <c r="D11" s="2">
+        <v>0.729768786127167</v>
+      </c>
+      <c r="E11" s="2">
+        <v>0.68644927855976701</v>
+      </c>
+      <c r="F11" s="2">
+        <v>0.39174628989631999</v>
+      </c>
+      <c r="H11" t="s">
+        <v>12</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A1:E1"/>
+  <mergeCells count="2">
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A7:F7"/>
   </mergeCells>
+  <conditionalFormatting sqref="B1:F1048576">
+    <cfRule type="colorScale" priority="1">
+      <colorScale>
+        <cfvo type="num" val="0"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="num" val="1"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Recalc results for single prompt grading with json-repair
</commit_message>
<xml_diff>
--- a/src/results/llm/single_prompt_testing_01/responses/results_for_presentation_single_prompt.xlsx
+++ b/src/results/llm/single_prompt_testing_01/responses/results_for_presentation_single_prompt.xlsx
@@ -8,12 +8,12 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\repos\Using-LLM-for-automated-feedback-generation-on-a-bachelor-thesis\src\results\llm\single_prompt_testing_01\responses\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8AE37CFA-752D-40AC-A8CF-ADFE1C4F1433}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{56E27BFD-F5F2-4DF9-8759-F3FE6F005CD9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="15" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Single_prompt" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="15">
   <si>
     <t>human1</t>
   </si>
@@ -75,6 +75,12 @@
   </si>
   <si>
     <t>percentage not parsed</t>
+  </si>
+  <si>
+    <t>gemma4-26b-q4 vs humanx after parsing with json-repair</t>
+  </si>
+  <si>
+    <t>Total of unparsed questions</t>
   </si>
 </sst>
 </file>
@@ -106,7 +112,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -114,19 +120,41 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="10" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="10" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -407,41 +435,41 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H11"/>
+  <dimension ref="A1:H18"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="20.7109375" style="2" customWidth="1"/>
-    <col min="3" max="3" width="16.42578125" style="2" customWidth="1"/>
-    <col min="4" max="4" width="14.7109375" style="2" customWidth="1"/>
-    <col min="5" max="5" width="11.7109375" style="2" customWidth="1"/>
-    <col min="6" max="6" width="13.28515625" style="2" customWidth="1"/>
+    <col min="2" max="2" width="20.7109375" style="1" customWidth="1"/>
+    <col min="3" max="3" width="16.42578125" style="1" customWidth="1"/>
+    <col min="4" max="4" width="14.7109375" style="1" customWidth="1"/>
+    <col min="5" max="5" width="11.7109375" style="1" customWidth="1"/>
+    <col min="6" max="6" width="13.28515625" style="1" customWidth="1"/>
     <col min="8" max="8" width="24.85546875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="B1" s="1"/>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
-      <c r="E1" s="1"/>
-      <c r="F1" s="1"/>
+      <c r="B1" s="3"/>
+      <c r="C1" s="3"/>
+      <c r="D1" s="3"/>
+      <c r="E1" s="3"/>
+      <c r="F1" s="3"/>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="B2" s="2" t="s">
+      <c r="B2" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="C2" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="D2" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="E2" s="2" t="s">
+      <c r="E2" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="F2" s="2" t="s">
+      <c r="F2" s="1" t="s">
         <v>7</v>
       </c>
     </row>
@@ -449,19 +477,19 @@
       <c r="A3" t="s">
         <v>0</v>
       </c>
-      <c r="B3" s="2">
+      <c r="B3" s="1">
         <v>0.86513994910941405</v>
       </c>
-      <c r="C3" s="2">
+      <c r="C3" s="1">
         <v>0.46703296703296698</v>
       </c>
-      <c r="D3" s="2">
+      <c r="D3" s="1">
         <v>0.60660124888492395</v>
       </c>
-      <c r="E3" s="2">
+      <c r="E3" s="1">
         <v>0.63510840476282804</v>
       </c>
-      <c r="F3" s="2">
+      <c r="F3" s="1">
         <v>0.32199138227499802</v>
       </c>
       <c r="H3" t="s">
@@ -472,22 +500,22 @@
       <c r="A4" t="s">
         <v>1</v>
       </c>
-      <c r="B4" s="2">
+      <c r="B4" s="1">
         <v>0.631043256997455</v>
       </c>
-      <c r="C4" s="2">
+      <c r="C4" s="1">
         <v>0.43508771929824502</v>
       </c>
-      <c r="D4" s="2">
+      <c r="D4" s="1">
         <v>0.515057113187954</v>
       </c>
-      <c r="E4" s="2">
+      <c r="E4" s="1">
         <v>0.59857688879275095</v>
       </c>
-      <c r="F4" s="2">
+      <c r="F4" s="1">
         <v>0.214548512561757</v>
       </c>
-      <c r="H4" s="3">
+      <c r="H4" s="2">
         <f>(37/64)*100</f>
         <v>57.8125</v>
       </c>
@@ -496,19 +524,19 @@
       <c r="A5" t="s">
         <v>2</v>
       </c>
-      <c r="B5" s="2">
+      <c r="B5" s="1">
         <v>0.87022900763358702</v>
       </c>
-      <c r="C5" s="2">
+      <c r="C5" s="1">
         <v>0.42857142857142799</v>
       </c>
-      <c r="D5" s="2">
+      <c r="D5" s="1">
         <v>0.57430730478589398</v>
       </c>
-      <c r="E5" s="2">
+      <c r="E5" s="1">
         <v>0.58288290299729795</v>
       </c>
-      <c r="F5" s="2">
+      <c r="F5" s="1">
         <v>0.24909747292418699</v>
       </c>
       <c r="H5" t="s">
@@ -516,29 +544,29 @@
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A7" s="1" t="s">
+      <c r="A7" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="B7" s="1"/>
-      <c r="C7" s="1"/>
-      <c r="D7" s="1"/>
-      <c r="E7" s="1"/>
-      <c r="F7" s="1"/>
+      <c r="B7" s="3"/>
+      <c r="C7" s="3"/>
+      <c r="D7" s="3"/>
+      <c r="E7" s="3"/>
+      <c r="F7" s="3"/>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="B8" s="2" t="s">
+      <c r="B8" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="C8" s="2" t="s">
+      <c r="C8" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D8" s="2" t="s">
+      <c r="D8" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="E8" s="2" t="s">
+      <c r="E8" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="F8" s="2" t="s">
+      <c r="F8" s="1" t="s">
         <v>7</v>
       </c>
     </row>
@@ -546,19 +574,19 @@
       <c r="A9" t="s">
         <v>0</v>
       </c>
-      <c r="B9" s="2">
+      <c r="B9" s="1">
         <v>0.83447098976109202</v>
       </c>
-      <c r="C9" s="2">
+      <c r="C9" s="1">
         <v>0.67170329670329598</v>
       </c>
-      <c r="D9" s="2">
+      <c r="D9" s="1">
         <v>0.74429223744292194</v>
       </c>
-      <c r="E9" s="2">
+      <c r="E9" s="1">
         <v>0.72187778240661304</v>
       </c>
-      <c r="F9" s="2">
+      <c r="F9" s="1">
         <v>0.451287120202845</v>
       </c>
       <c r="H9" t="s">
@@ -569,22 +597,22 @@
       <c r="A10" t="s">
         <v>1</v>
       </c>
-      <c r="B10" s="2">
+      <c r="B10" s="1">
         <v>0.639931740614334</v>
       </c>
-      <c r="C10" s="2">
+      <c r="C10" s="1">
         <v>0.65789473684210498</v>
       </c>
-      <c r="D10" s="2">
+      <c r="D10" s="1">
         <v>0.64878892733563998</v>
       </c>
-      <c r="E10" s="2">
+      <c r="E10" s="1">
         <v>0.66530355457691004</v>
       </c>
-      <c r="F10" s="2">
+      <c r="F10" s="1">
         <v>0.330723263960436</v>
       </c>
-      <c r="H10" s="3">
+      <c r="H10" s="2">
         <f>(20/64)*100</f>
         <v>31.25</v>
       </c>
@@ -593,31 +621,126 @@
       <c r="A11" t="s">
         <v>2</v>
       </c>
-      <c r="B11" s="2">
+      <c r="B11" s="1">
         <v>0.86177474402730303</v>
       </c>
-      <c r="C11" s="2">
+      <c r="C11" s="1">
         <v>0.63283208020050097</v>
       </c>
-      <c r="D11" s="2">
+      <c r="D11" s="1">
         <v>0.729768786127167</v>
       </c>
-      <c r="E11" s="2">
+      <c r="E11" s="1">
         <v>0.68644927855976701</v>
       </c>
-      <c r="F11" s="2">
+      <c r="F11" s="1">
         <v>0.39174628989631999</v>
       </c>
       <c r="H11" t="s">
         <v>12</v>
       </c>
     </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A14" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="B14" s="5"/>
+      <c r="C14" s="5"/>
+      <c r="D14" s="5"/>
+      <c r="E14" s="5"/>
+      <c r="F14" s="5"/>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A15" s="6"/>
+      <c r="B15" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="C15" s="7" t="s">
+        <v>4</v>
+      </c>
+      <c r="D15" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="E15" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="F15" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="H15" s="4" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A16" s="6" t="s">
+        <v>0</v>
+      </c>
+      <c r="B16" s="8">
+        <v>0.82063305978898005</v>
+      </c>
+      <c r="C16" s="8">
+        <v>0.96153846153846101</v>
+      </c>
+      <c r="D16" s="8">
+        <v>0.88551549652118899</v>
+      </c>
+      <c r="E16" s="8">
+        <v>0.83641227234990101</v>
+      </c>
+      <c r="F16" s="8">
+        <v>0.676580537465027</v>
+      </c>
+      <c r="H16">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A17" s="6" t="s">
+        <v>1</v>
+      </c>
+      <c r="B17" s="8">
+        <v>0.64009378663540395</v>
+      </c>
+      <c r="C17" s="8">
+        <v>0.95789473684210502</v>
+      </c>
+      <c r="D17" s="8">
+        <v>0.76739283204497499</v>
+      </c>
+      <c r="E17" s="8">
+        <v>0.71967263009582705</v>
+      </c>
+      <c r="F17" s="8">
+        <v>0.46896620876366102</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A18" s="6" t="s">
+        <v>2</v>
+      </c>
+      <c r="B18" s="8">
+        <v>0.86869871043376301</v>
+      </c>
+      <c r="C18" s="8">
+        <v>0.92857142857142805</v>
+      </c>
+      <c r="D18" s="8">
+        <v>0.89763779527558996</v>
+      </c>
+      <c r="E18" s="8">
+        <v>0.84062427535866502</v>
+      </c>
+      <c r="F18" s="8">
+        <v>0.68199459014465402</v>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="2">
+  <mergeCells count="3">
     <mergeCell ref="A1:F1"/>
     <mergeCell ref="A7:F7"/>
+    <mergeCell ref="A14:F14"/>
   </mergeCells>
-  <conditionalFormatting sqref="B1:F1048576">
+  <conditionalFormatting sqref="B1:F1048576 H15">
     <cfRule type="colorScale" priority="1">
       <colorScale>
         <cfvo type="num" val="0"/>

</xml_diff>

<commit_message>
Metrics for single prompt with structured output json-repair
</commit_message>
<xml_diff>
--- a/src/results/llm/single_prompt_testing_01/responses/results_for_presentation_single_prompt.xlsx
+++ b/src/results/llm/single_prompt_testing_01/responses/results_for_presentation_single_prompt.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\repos\Using-LLM-for-automated-feedback-generation-on-a-bachelor-thesis\src\results\llm\single_prompt_testing_01\responses\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3FC31A5F-E1BA-4AF4-A717-F9E72735AF1A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1ED540BA-C699-4768-8DAA-3C7DC30C17B6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="15" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Single_prompt" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="18">
   <si>
     <t>human1</t>
   </si>
@@ -87,6 +87,9 @@
   </si>
   <si>
     <t>20 JSONs which is</t>
+  </si>
+  <si>
+    <t>gemma4-26b-q4 vs humanx WITH STRUCTURED OUTPUT (parsing with json-repair)</t>
   </si>
 </sst>
 </file>
@@ -158,7 +161,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -177,13 +180,22 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Neutral" xfId="1" builtinId="28"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="3">
+  <dxfs count="4">
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -206,11 +218,11 @@
     </dxf>
     <dxf>
       <font>
-        <color rgb="FF006100"/>
+        <color rgb="FF9C0006"/>
       </font>
       <fill>
         <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
+          <bgColor rgb="FFFFC7CE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -490,7 +502,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:P18"/>
+  <dimension ref="A1:P24"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="20.7109375" style="1" customWidth="1"/>
@@ -564,7 +576,7 @@
       <c r="K3" t="s">
         <v>0</v>
       </c>
-      <c r="L3" s="10">
+      <c r="L3" s="1">
         <v>0.87275111483504597</v>
       </c>
     </row>
@@ -594,7 +606,7 @@
       <c r="K4" t="s">
         <v>1</v>
       </c>
-      <c r="L4" s="10">
+      <c r="L4" s="1">
         <v>0.76214905902143104</v>
       </c>
     </row>
@@ -623,7 +635,7 @@
       <c r="K5" t="s">
         <v>2</v>
       </c>
-      <c r="L5" s="10">
+      <c r="L5" s="1">
         <v>0.83914274034009595</v>
       </c>
     </row>
@@ -787,7 +799,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A17" s="4" t="s">
         <v>1</v>
       </c>
@@ -811,7 +823,7 @@
         <v>0.46896620876366102</v>
       </c>
     </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A18" s="4" t="s">
         <v>2</v>
       </c>
@@ -835,14 +847,171 @@
         <v>0.68199459014465402</v>
       </c>
     </row>
+    <row r="20" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A20" s="8" t="s">
+        <v>17</v>
+      </c>
+      <c r="B20" s="8"/>
+      <c r="C20" s="8"/>
+      <c r="D20" s="8"/>
+      <c r="E20" s="8"/>
+      <c r="F20" s="8"/>
+      <c r="G20" s="8"/>
+      <c r="I20" s="3" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="21" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A21" s="4"/>
+      <c r="B21" s="5" t="s">
+        <v>3</v>
+      </c>
+      <c r="C21" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="D21" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="E21" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="F21" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="G21" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="I21">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="22" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A22" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="B22" s="1">
+        <v>0.82084309133489397</v>
+      </c>
+      <c r="C22" s="1">
+        <v>0.96291208791208704</v>
+      </c>
+      <c r="D22" s="1">
+        <v>0.88621997471554903</v>
+      </c>
+      <c r="E22" s="1">
+        <v>0.83722763441659798</v>
+      </c>
+      <c r="F22" s="6">
+        <f>E22-L3</f>
+        <v>-3.5523480418447995E-2</v>
+      </c>
+      <c r="G22" s="1">
+        <v>0.67825391598852203</v>
+      </c>
+    </row>
+    <row r="23" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A23" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="B23" s="1">
+        <v>0.64051522248243498</v>
+      </c>
+      <c r="C23" s="1">
+        <v>0.95964912280701697</v>
+      </c>
+      <c r="D23" s="1">
+        <v>0.76825842696629199</v>
+      </c>
+      <c r="E23" s="1">
+        <v>0.72043873729266905</v>
+      </c>
+      <c r="F23" s="6">
+        <f t="shared" ref="F23:F24" si="1">E23-L4</f>
+        <v>-4.171032172876199E-2</v>
+      </c>
+      <c r="G23" s="1">
+        <v>0.47062362141567998</v>
+      </c>
+    </row>
+    <row r="24" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A24" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="B24" s="1">
+        <v>0.86885245901639296</v>
+      </c>
+      <c r="C24" s="1">
+        <v>0.929824561403508</v>
+      </c>
+      <c r="D24" s="1">
+        <v>0.89830508474576198</v>
+      </c>
+      <c r="E24" s="1">
+        <v>0.84146023468057296</v>
+      </c>
+      <c r="F24" s="6">
+        <f t="shared" si="1"/>
+        <v>2.317494340477011E-3</v>
+      </c>
+      <c r="G24" s="1">
+        <v>0.68369028006589705</v>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="4">
+  <mergeCells count="5">
     <mergeCell ref="A1:G1"/>
     <mergeCell ref="A7:G7"/>
     <mergeCell ref="A14:G14"/>
     <mergeCell ref="K2:P2"/>
+    <mergeCell ref="A20:G20"/>
   </mergeCells>
   <conditionalFormatting sqref="B1:E1048576 I15 G1:G1048576">
+    <cfRule type="colorScale" priority="9">
+      <colorScale>
+        <cfvo type="num" val="0"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="num" val="1"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F16:F17">
+    <cfRule type="cellIs" dxfId="3" priority="4" operator="lessThan">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F16:F18">
+    <cfRule type="cellIs" dxfId="2" priority="5" operator="greaterThan">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="L3">
+    <cfRule type="colorScale" priority="8">
+      <colorScale>
+        <cfvo type="num" val="0"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="num" val="1"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="L4">
+    <cfRule type="colorScale" priority="7">
+      <colorScale>
+        <cfvo type="num" val="0"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="num" val="1"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="L5">
     <cfRule type="colorScale" priority="6">
       <colorScale>
         <cfvo type="num" val="0"/>
@@ -854,31 +1023,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="L3">
-    <cfRule type="colorScale" priority="5">
-      <colorScale>
-        <cfvo type="num" val="0"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="num" val="1"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="L4">
-    <cfRule type="colorScale" priority="4">
-      <colorScale>
-        <cfvo type="num" val="0"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="num" val="1"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="L5">
+  <conditionalFormatting sqref="I20">
     <cfRule type="colorScale" priority="3">
       <colorScale>
         <cfvo type="num" val="0"/>
@@ -890,13 +1035,13 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F16:F18">
-    <cfRule type="cellIs" dxfId="2" priority="2" operator="greaterThan">
+  <conditionalFormatting sqref="F22:F24">
+    <cfRule type="cellIs" dxfId="1" priority="1" operator="lessThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F16:F17">
-    <cfRule type="cellIs" dxfId="0" priority="1" operator="lessThan">
+  <conditionalFormatting sqref="F22:F24">
+    <cfRule type="cellIs" dxfId="0" priority="2" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>